<commit_message>
update patientId + uniformisation id 4b43dd6a99bc06edacd1b56520975081ffc550a7
</commit_message>
<xml_diff>
--- a/spec-tech/ig/StructureDefinition-pdlgcFournisseurSortant.xlsx
+++ b/spec-tech/ig/StructureDefinition-pdlgcFournisseurSortant.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-23T14:32:10+00:00</t>
+    <t>2026-07-23T16:03:49+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -3230,7 +3230,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="24" hidden="true">
+    <row r="24">
       <c r="A24" t="s" s="2">
         <v>156</v>
       </c>
@@ -3249,7 +3249,7 @@
         <v>79</v>
       </c>
       <c r="H24" t="s" s="2">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="I24" t="s" s="2">
         <v>73</v>

</xml_diff>